<commit_message>
Schedule tags [BRING LAPTOP] days from one LAPTOP_DAYS list; checklists repeat it
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015RAcPZi5nkqZkcCQ9LAREd
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
@@ -571,7 +571,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Newton's laws</t>
+          <t>Newton's laws [BRING LAPTOP]</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -1936,7 +1936,7 @@
       <c r="F43" s="2" t="inlineStr"/>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Log into posit.smith.edu and open the driven-pendulum notebook on Moodle; bring your laptop</t>
+          <t>Log into jupyterhub.smith.edu and open the driven-pendulum notebook on Moodle; bring your laptop</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Review 2026-09-19: HW01/HW02 Friday dates recorded, Mountain Day rule un-inverted, two-star budget guard, stale grading/attendance-cap text fixed
- make_fall2026_calendar.py: HW01 Fri Sep 18, HW02 Fri Sep 25 (match live
  Moodle; HW03+ Wednesday pending decision); 2.42 bracket no longer claims
  2.41 was done in class; Mountain Day holder text follows TODO item 6.
- make_active_learning.py: warn when a (**) problem has < 20 Active min.
- TODO.md: attendance caps are IN (commit 18bd029), HW due-day state,
  Mountain Day after-Oct-5 gap, Moodle rebuild marked done.
- README.md, MoodleBuildSpec.md: HW due state; Taylor scan and ISM PDFs are
  posted (TODO item 10); calendar embed is a label.
- PHY317Syllabus.tex/.pdf: 70 -> 112 participation points.
- Regenerated xlsx.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
@@ -665,11 +665,7 @@
           <t>2.25</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>HW01</t>
-        </is>
-      </c>
+      <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
@@ -706,7 +702,11 @@
           <t>2.49</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>HW01</t>
+        </is>
+      </c>
       <c r="I6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
@@ -778,11 +778,7 @@
           <t>3.16</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>HW02</t>
-        </is>
-      </c>
+      <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
@@ -818,7 +814,11 @@
           <t>3.32</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>HW02</t>
+        </is>
+      </c>
       <c r="I9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
@@ -947,14 +947,14 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Mountain Day holder (if Mountain Day has already happened: Ch 1-4 problem session)</t>
+          <t>Mountain Day holder (if no class was lost to Mountain Day: Ch 1-4 problem session)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Bring one Ch 1-4 problem you want worked in the problem session (skip if Mountain Day)</t>
+          <t>Bring one Ch 1-4 problem you want worked in the problem session (skip if this slot absorbed a Mountain Day class)</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Wed Sep 16</t>
+          <t>Fri Sep 18</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Wed Sep 23</t>
+          <t>Fri Sep 25</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2.14 [look up the integral], 2.31, 2.36, 2.39, 2.42 [2.41 done in class], 2.53</t>
+          <t>2.14 [look up the integral], 2.31, 2.36, 2.39, 2.42 [2.41 is in the posted Ch 2 in-class solutions; read back in class Mon Sep 21], 2.53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
HW due Fridays from HW02 on (decided with the class 2026-09-19)
HW03 Fri Oct 2, HW05 Fri Oct 16, HW07 Fri Oct 30, HW10 Fri Nov 20, HW13
Fri Dec 18; HW04 Mon Oct 5, HW08 Wed Nov 4, HW11 Mon Nov 23 stay. Syllabus
line and PDF, spec, README, TODO updated; xlsx regenerated. Moodle edits
for HW03/05/07/10/13 still by hand (TODO).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
@@ -890,11 +890,7 @@
           <t>4.31</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>HW03</t>
-        </is>
-      </c>
+      <c r="H11" s="2" t="inlineStr"/>
       <c r="I11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
@@ -930,7 +926,11 @@
           <t>4.41</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>HW03</t>
+        </is>
+      </c>
       <c r="I12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
@@ -1125,11 +1125,7 @@
           <t>5.21</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>HW05</t>
-        </is>
-      </c>
+      <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1164,7 +1160,11 @@
           <t>5.35</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>HW05</t>
+        </is>
+      </c>
       <c r="I19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
@@ -1335,11 +1335,7 @@
           <t>7.1</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>HW07</t>
-        </is>
-      </c>
+      <c r="H24" s="2" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
@@ -1370,7 +1366,11 @@
           <t>Read 7.2-7.3: in a sentence, what makes a constraint holonomic? Give one example of each kind</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>HW07</t>
+        </is>
+      </c>
       <c r="I25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
@@ -1639,11 +1639,7 @@
           <t>9.7</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>HW10</t>
-        </is>
-      </c>
+      <c r="H33" s="2" t="inlineStr"/>
       <c r="I33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
@@ -1674,7 +1670,11 @@
           <t>9.12</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>HW10</t>
+        </is>
+      </c>
       <c r="I34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
@@ -1974,7 +1974,7 @@
       <c r="B45" s="4" t="n"/>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Wed Dec 16</t>
+          <t>Fri Dec 18</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -2132,7 +2132,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Wed Sep 30</t>
+          <t>Fri Oct 2</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Wed Oct 14</t>
+          <t>Fri Oct 16</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Wed Oct 28</t>
+          <t>Fri Oct 30</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Wed Nov 18</t>
+          <t>Fri Nov 20</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Wed Dec 16</t>
+          <t>Fri Dec 18</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Calendar: a graced set is just listed on both dates
The "- or Mon Oct 19, no penalty" / "- extended from Fri Oct 16" suffixes
wrapped to three lines in a narrow column. Moodle carries which date is
the deadline (Due vs Cut-off); the calendar only needs to show both.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
@@ -1150,7 +1150,7 @@
       <c r="G19" s="4" t="inlineStr"/>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>HW05 (Ch 5) - or Mon Oct 19, no penalty</t>
+          <t>HW05 (Ch 5)</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>HW05 (Ch 5) - extended from Fri Oct 16</t>
+          <t>HW05 (Ch 5)</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Calendar: HW13 due Mon Dec 14, the last class day
Was Fri Dec 18, in reading period (Michael, 2026-09-24). Will's HW13 was
Thu Dec 11, also his last week rather than reading period, so this is
closer to his. Nothing is now due on a non-class day, so the generated
"Reading period" row -- which existed only to carry HW13 -- is gone and
the Moodle chunk-2 embed range shrinks to A17:I45.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1962,7 +1962,11 @@
           <t>Bring one question for the final-exam review</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>HW13 (Ch 12)</t>
+        </is>
+      </c>
       <c r="I44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
@@ -1970,42 +1974,19 @@
       <c r="B45" s="3" t="n"/>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Fri Dec 18</t>
+          <t>Sat Dec 19</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Reading period</t>
+          <t>Final exam period Dec 19-22 (self-scheduled)</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr"/>
       <c r="F45" s="3" t="inlineStr"/>
       <c r="G45" s="3" t="inlineStr"/>
-      <c r="H45" s="3" t="inlineStr">
-        <is>
-          <t>HW13 (Ch 12)</t>
-        </is>
-      </c>
-      <c r="I45" s="3" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="3" t="n"/>
-      <c r="B46" s="3" t="n"/>
-      <c r="C46" s="3" t="inlineStr">
-        <is>
-          <t>Sat Dec 19</t>
-        </is>
-      </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>Final exam period Dec 19-22 (self-scheduled)</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr"/>
-      <c r="F46" s="3" t="inlineStr"/>
-      <c r="G46" s="3" t="inlineStr"/>
-      <c r="H46" s="3" t="inlineStr"/>
-      <c r="I46" s="3" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr"/>
+      <c r="I45" s="3" t="inlineStr">
         <is>
           <t>Final (Ch 12 required + optional grade-replacement)</t>
         </is>
@@ -2398,7 +2379,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Fri Dec 18</t>
+          <t>Mon Dec 14</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Generators: checklist wording and guards, calendar comments, answer-sheet crops, brachistochrone times (DRY A3, A4, A7, A11)
Checklists: in-class line reads the pack's notes through packnotes.layout(),
EXAM DAY instrument line, HW_GRACE and EXTRA_DUE lines, header fixed,
class_rows asserts counts and exam placement. Calendar: superseded
due-date comments marked as history, docstring and participation FLAG
match 210's; chapter slides guard a chapter with no class days; TODO
embed range A17:I45. Answer sheets: PIL at top, anchored render_pages
regex with the full slug. audit_taylor_coverage scans to PDF page 538 so
Ch 12 problems are seen. brachistochrone.pdf regenerated with the closed
forms (straight line 0.992 s, cycloid 1.010 s were wrong in the 2nd-3rd
decimal). PHY317 F2026 Calendar.xlsx regenerated: two cells (Dec 11
laptop tag, HW09 covers 7.10) catch up with generator edits made since
the file was last written.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
@@ -1921,7 +1921,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Chaos: sensitivity to initial conditions; Liouville aside</t>
+          <t>Chaos: sensitivity to initial conditions; Liouville aside [BRING LAPTOP]</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2276,7 +2276,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>7.5, 7.8, 7.9, 8.1-8.2: Lagrangian examples; Noether; multipliers; two-body setup</t>
+          <t>7.5, 7.8, 7.10, 8.1-8.2: Lagrangian examples; Noether; multipliers; two-body setup</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">

</xml_diff>

<commit_message>
317 calendar: the three flex days move to the end of term (Dec 9, 11, 14: flex OR Noether OR Jarzynski), content bumped forward, PCCIs re-keyed, laptop day Dec 4; course map and schedule colour flex days lilac (Michael, 2026-10-08)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
@@ -32,7 +32,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +52,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDE9FE"/>
       </patternFill>
     </fill>
   </fills>
@@ -81,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -93,6 +98,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1559,14 +1567,22 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Catch-up / review day (Exam 2 is Monday)</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr"/>
-      <c r="F31" s="2" t="inlineStr"/>
+          <t>Angular velocity; rotating frames</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>9.3-9.5</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Math Methods: Ch. 8 (Vectors in Curvilinear Coordinates)</t>
+        </is>
+      </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Bring one Ch 5-7 problem you want worked in review</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1617,22 +1633,18 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Angular velocity; rotating frames</t>
+          <t>Centrifugal force; Coriolis force</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>9.3-9.5</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>Math Methods: Ch. 8 (Vectors in Curvilinear Coordinates)</t>
-        </is>
-      </c>
+          <t>9.6-9.8</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>9.12</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr"/>
@@ -1652,18 +1664,24 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Centrifugal force; Coriolis force</t>
+          <t>Coupled oscillators; two masses and three springs</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>9.6-9.8</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr"/>
+          <t>11.1-11.2</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Knight: Ch. 15 (Oscillations)
+Math Methods: Ch. 6 (Eigenvectors/Eigenvalues)
+Review the ideas behind basis vectors</t>
+        </is>
+      </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>9.12</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1687,24 +1705,22 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Coupled oscillators; two masses and three springs</t>
+          <t>Normal coordinates; weakly coupled oscillators; start the double pendulum</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>11.1-11.2</t>
+          <t>11.2-11.4</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Knight: Ch. 15 (Oscillations)
-Math Methods: Ch. 6 (Eigenvectors/Eigenvalues)
-Review the ideas behind basis vectors</t>
+          <t>Math Methods: Ch. 6 (Eigenvectors/Eigenvalues)</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>Read 11.3: in a sentence or two, what happens to the energy of two weakly coupled pendulums over time?</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr"/>
@@ -1762,22 +1778,18 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Normal coordinates; weakly coupled oscillators; start the double pendulum</t>
+          <t>Double pendulum</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>11.2-11.4</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>Math Methods: Ch. 6 (Eigenvectors/Eigenvalues)</t>
-        </is>
-      </c>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Read 11.3: in a sentence or two, what happens to the energy of two weakly coupled pendulums over time?</t>
+          <t>Write down the Lagrangian of a simple pendulum (length L, angle phi); no need to solve it</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -1801,18 +1813,18 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Double pendulum</t>
+          <t>Chaos: the driven damped pendulum; period doubling</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>12.1-12.4</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr"/>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Write down the Lagrangian of a simple pendulum (length L, angle phi); no need to solve it</t>
+          <t>Read 12.1-12.2: in a sentence, what does it mean for an equation of motion to be linear, and what do we lose when it isn't?</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -1832,14 +1844,18 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Catch-up / review day (Exam 3 is Monday)</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr"/>
+          <t>Chaos: sensitivity to initial conditions; Liouville aside [BRING LAPTOP]</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>12.4-12.5</t>
+        </is>
+      </c>
       <c r="F40" s="2" t="inlineStr"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Bring one Ch 8, 9, or 11 problem you want worked in review</t>
+          <t>Log into jupyterhub.smith.edu and open the driven-pendulum notebook on Moodle; bring your laptop</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -1877,97 +1893,81 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="B42" s="2" t="n">
+      <c r="B42" s="5" t="n">
         <v>36</v>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C42" s="5" t="inlineStr">
         <is>
           <t>Wed Dec 9</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>Chaos: the driven damped pendulum; period doubling</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>12.1-12.4</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>Read 12.1-12.2: in a sentence, what does it mean for an equation of motion to be linear, and what do we lose when it isn't?</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr"/>
-      <c r="I42" s="2" t="inlineStr"/>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Flex day: Noether's theorem (Taylor 7.8) OR Jarzynski OR catch-up</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr"/>
+      <c r="F42" s="5" t="inlineStr"/>
+      <c r="G42" s="5" t="inlineStr"/>
+      <c r="H42" s="5" t="inlineStr"/>
+      <c r="I42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="A43" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="B43" s="2" t="n">
+      <c r="B43" s="5" t="n">
         <v>37</v>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C43" s="5" t="inlineStr">
         <is>
           <t>Fri Dec 11</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>Chaos: sensitivity to initial conditions; Liouville aside [BRING LAPTOP]</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>12.4-12.5</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr"/>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>Log into jupyterhub.smith.edu and open the driven-pendulum notebook on Moodle; bring your laptop</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr"/>
-      <c r="I43" s="2" t="inlineStr"/>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Flex day: Noether's theorem (Taylor 7.8) OR Jarzynski OR catch-up</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr"/>
+      <c r="F43" s="5" t="inlineStr"/>
+      <c r="G43" s="5" t="inlineStr"/>
+      <c r="H43" s="5" t="inlineStr"/>
+      <c r="I43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="A44" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B44" s="2" t="n">
+      <c r="B44" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C44" s="5" t="inlineStr">
         <is>
           <t>Mon Dec 14</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>Last day: review and wrap-up</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="2" t="inlineStr"/>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Last day: flex (Noether OR Jarzynski OR wrap-up)</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr"/>
+      <c r="F44" s="5" t="inlineStr"/>
+      <c r="G44" s="5" t="inlineStr">
         <is>
           <t>Bring one question for the final-exam review</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="H44" s="5" t="inlineStr">
         <is>
           <t>HW13 (Ch 12)</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr"/>
+      <c r="I44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n"/>
@@ -2014,34 +2014,34 @@
   </cols>
   <sheetData>
     <row r="1" ht="45" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>All problems from Taylor, Classical Mechanics (2005). Due FRIDAYS at 10:00 PM on Moodle from HW02 on (decided with the class 2026-09-19) unless the Due column says otherwise -- the exceptions sit right before an exam or a break. Custom problems are written out in full on the Moodle assignment page.</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>HW</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Covers</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>Chapters</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>Problems</t>
         </is>
@@ -2423,27 +2423,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>Number</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>Drop</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>Points Each</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>Total Points</t>
         </is>
@@ -2562,266 +2562,266 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Chapter</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>Look at (PCCI source)</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>In class</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="n">
+      <c r="A2" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Day 1</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>1.4, 1.6, 1.10, 1.11, 1.31, 1.35</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>1.9, 1.18, 1.26, 1.43, 1.47, 1.48</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>HW01: 1.27, 1.45, 1.46, 1.49, 1.50 (computational)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Day 1</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>2.1, 2.5, 2.7</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>2.4, 2.11, 2.12, 2.13</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>HW02: 2.14, 2.31, 2.36, 2.39, 2.42, 2.53</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="A4" s="6" t="n"/>
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Day 2</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>2.16, 2.25</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>2.33, 2.34, 2.35, 2.41</t>
         </is>
       </c>
-      <c r="E4" s="5" t="n"/>
+      <c r="E4" s="6" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n"/>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="n"/>
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Day 3</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>2.49</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>2.52, 2.54</t>
         </is>
       </c>
-      <c r="E5" s="5" t="n"/>
+      <c r="E5" s="6" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Day 1</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>3.7</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>3.5, 3.10, 3.11</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>HW03: 3.8, 3.13, 3.19, 3.35, 3.36, chain lifted at constant speed (optional challenge)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Day 2</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>3.16, 3.17, 3.25</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>3.21, 3.27</t>
         </is>
       </c>
-      <c r="E7" s="5" t="n"/>
+      <c r="E7" s="6" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Day 3</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>3.32</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>3.29, 3.34</t>
         </is>
       </c>
-      <c r="E8" s="5" t="n"/>
+      <c r="E8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Day 1</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>4.7, 4.16</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>4.2, 4.3, 4.12, 4.15</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>HW04: 4.4, 4.8, 4.13 (optional), 4.24(a-c), Variation of gravity with height, 4.36, 4.39 (advanced, optional), 4.53</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Day 2</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>4.31</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>4.23, 4.26, 4.28</t>
         </is>
       </c>
-      <c r="E10" s="5" t="n"/>
+      <c r="E10" s="6" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Day 3</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>4.41</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>4.46, 4.48</t>
         </is>
       </c>
-      <c r="E11" s="5" t="n"/>
+      <c r="E11" s="6" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n">
+      <c r="A12" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Day 1</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>5.1, 5.3</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>5.6, 5.8, 5.12</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>HW05: 5.4, 5.7, 5.13
 HW06: 5.28, 5.32 (optional), 5.43, RLC circuit as an SHO, Square-wave drive (or 5.49)</t>
@@ -2829,82 +2829,82 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Day 2</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>5.21</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>5.22, 5.26</t>
         </is>
       </c>
-      <c r="E13" s="5" t="n"/>
+      <c r="E13" s="6" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n"/>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Day 3</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>5.35</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>5.40, 5.41, 5.42, 5.44</t>
         </is>
       </c>
-      <c r="E14" s="5" t="n"/>
+      <c r="E14" s="6" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Day 4</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>5.47</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>5.49</t>
         </is>
       </c>
-      <c r="E15" s="5" t="n"/>
+      <c r="E15" s="6" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n">
+      <c r="A16" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Day 1</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>6.3, 6.4</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>6.1, 6.2</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>HW07: 6.7, 6.11, 6.14, 6.17, Brachistochrone revisited
 HW08: 6.23, 6.24 (advanced, optional), 6.27</t>
@@ -2912,63 +2912,63 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Day 2</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>6.8</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>6.9, 6.18</t>
         </is>
       </c>
-      <c r="E17" s="5" t="n"/>
+      <c r="E17" s="6" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n"/>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Day 3</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>6.20</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>6.21, 6.25</t>
         </is>
       </c>
-      <c r="E18" s="5" t="n"/>
+      <c r="E18" s="6" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="n">
+      <c r="A19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Day 1</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>7.1, 7.2</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>7.4, 7.8</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>HW08: 7.3, 7.10, 7.14
 HW09: 7.27, 7.31, 7.34, 7.38 (optional challenge), 7.46 (Noether)</t>
@@ -2976,59 +2976,59 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="n"/>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Day 2</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr"/>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr"/>
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>7.9</t>
         </is>
       </c>
-      <c r="E20" s="5" t="n"/>
+      <c r="E20" s="6" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="n"/>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>Day 3</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>7.17, 7.19</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>7.20, 7.33, 7.36</t>
         </is>
       </c>
-      <c r="E21" s="5" t="n"/>
+      <c r="E21" s="6" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="n">
+      <c r="A22" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Day 1</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>8.6, 8.8</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>8.3, 8.10</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>HW09: 8.2
 HW10: 8.9, 8.13, 8.14 (optional challenge), 8.15, 8.18, 8.23
@@ -3037,192 +3037,192 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="n"/>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>Day 2</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>8.19, 8.20</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>8.12, 8.21</t>
         </is>
       </c>
-      <c r="E23" s="5" t="n"/>
+      <c r="E23" s="6" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="n"/>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="A24" s="6" t="n"/>
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Day 3</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>8.28, 8.32</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>8.29, 8.33, 8.34</t>
         </is>
       </c>
-      <c r="E24" s="5" t="n"/>
+      <c r="E24" s="6" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="n">
+      <c r="A25" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>Day 1</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>9.1</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>9.2</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>HW11: 9.3, 9.9, 9.15, 9.17, 9.28, 9.29 (optional challenge)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="n"/>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="A26" s="6" t="n"/>
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>Day 2</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>9.7</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>9.8</t>
         </is>
       </c>
-      <c r="E26" s="5" t="n"/>
+      <c r="E26" s="6" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="n"/>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="A27" s="6" t="n"/>
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>Day 3</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>9.12, 9.13</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>9.14, 9.16, 9.19</t>
         </is>
       </c>
-      <c r="E27" s="5" t="n"/>
+      <c r="E27" s="6" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="n">
+      <c r="A28" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Day 1</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>11.1</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>11.2, 11.3</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>HW12: 11.6, 11.9, 11.12, 11.14, 11.17 (optional)</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="n"/>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="A29" s="6" t="n"/>
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>Day 2</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr"/>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr"/>
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>11.5</t>
         </is>
       </c>
-      <c r="E29" s="5" t="n"/>
+      <c r="E29" s="6" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="n"/>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="A30" s="6" t="n"/>
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>Day 3</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr"/>
-      <c r="D30" s="5" t="inlineStr"/>
-      <c r="E30" s="5" t="n"/>
+      <c r="C30" s="6" t="inlineStr"/>
+      <c r="D30" s="6" t="inlineStr"/>
+      <c r="E30" s="6" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="n">
+      <c r="A31" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>Day 1</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr"/>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr"/>
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>driven-pendulum notebook: period exploration, Poincare section</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>HW13: 12.1, 12.6, 12.7, 12.8-12.10 (optional), 12.13 + parts (b), (c)</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="n"/>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="A32" s="6" t="n"/>
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>Day 2</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr"/>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr"/>
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>bifurcation diagram, Lyapunov exponent</t>
         </is>
       </c>
-      <c r="E32" s="5" t="n"/>
+      <c r="E32" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Calendar: one-day slip after class 16 (Mon Oct 19 = Exam 1 hand-back + revision time)
Class 16's Fourier content finishes Wed Oct 21 (new class 17); everything after
moves one meeting later; the Dec 9 flex day is consumed (two flex days left).
PCCIs follow their topics (6.3 now due Fri Oct 23). Homework due dates unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
@@ -1220,24 +1220,20 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Calculus of variations; Fermat's principle; Euler-Lagrange</t>
+          <t>Fourier series analysis of driven SHO (continued)</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>6.1-6.2</t>
+          <t>5.7-5.8</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Math Methods: Ch. 4 (Partial Derivatives), Ch. 5 (Integration)</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>6.3</t>
-        </is>
-      </c>
+          <t>Math Methods: Ch. 9 (Fourier Series and Transforms)</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
       <c r="H21" s="2" t="inlineStr"/>
       <c r="I21" s="2" t="inlineStr"/>
     </row>
@@ -1255,22 +1251,22 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Euler-Lagrange equation; brachistochrone problem</t>
+          <t>Calculus of variations; Fermat's principle; Euler-Lagrange</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
+          <t>6.1-6.2</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Math Methods: Ch. 4 (Partial Derivatives), Ch. 5 (Integration)</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
           <t>6.3</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Math Methods: Ch. 4 (Partial Derivatives)</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>6.8</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1294,18 +1290,22 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Multiple variables; generalized coordinates</t>
+          <t>Euler-Lagrange equation; brachistochrone problem</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>6.4</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr"/>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Math Methods: Ch. 4 (Partial Derivatives)</t>
+        </is>
+      </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>6.20</t>
+          <t>6.8</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -1325,18 +1325,18 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Lagrange's equations; Hamilton's principle</t>
+          <t>Multiple variables; generalized coordinates</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.4</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.20</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -1356,18 +1356,18 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Constrained systems; generalized coordinates</t>
+          <t>Lagrange's equations; Hamilton's principle</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>7.2-7.3</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Read 7.2-7.3: in a sentence, what makes a constraint holonomic? Give one example of each kind</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1391,18 +1391,18 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Examples of Lagrange's equations; Noether's theorem (symmetries and conservation laws); Lagrange multipliers</t>
+          <t>Constrained systems; generalized coordinates</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>7.5, 7.8, 7.10</t>
+          <t>7.2-7.3</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>7.17</t>
+          <t>Read 7.2-7.3: in a sentence, what makes a constraint holonomic? Give one example of each kind</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -1422,22 +1422,18 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Central forces; reduced mass; equations of motion</t>
+          <t>Examples of Lagrange's equations; Noether's theorem (symmetries and conservation laws); Lagrange multipliers</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>8.1-8.4</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Knight: Ch. 12 (Gravity)</t>
-        </is>
-      </c>
+          <t>7.5, 7.8, 7.10</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>8.6</t>
+          <t>7.17</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -1457,23 +1453,22 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Orbits</t>
+          <t>Central forces; reduced mass; equations of motion</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>8.5-8.6</t>
+          <t>8.1-8.4</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Math Methods: Ch. 1 (ODEs)
-Calculus I &amp; II</t>
+          <t>Knight: Ch. 12 (Gravity)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>8.19</t>
+          <t>8.6</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1497,22 +1492,23 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Changing orbits</t>
+          <t>Orbits</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>8.7-8.8</t>
+          <t>8.5-8.6</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Calculus I &amp; II</t>
+          <t>Math Methods: Ch. 1 (ODEs)
+Calculus I &amp; II</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>8.28</t>
+          <t>8.19</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -1532,22 +1528,22 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Accelerating frames; tides</t>
+          <t>Changing orbits</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>9.1-9.2</t>
+          <t>8.7-8.8</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Math Methods: Ch. 8 (Vector Calculus)</t>
+          <t>Calculus I &amp; II</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>8.28</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -1567,22 +1563,22 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Angular velocity; rotating frames</t>
+          <t>Accelerating frames; tides</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>9.3-9.5</t>
+          <t>9.1-9.2</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Math Methods: Ch. 8 (Vectors in Curvilinear Coordinates)</t>
+          <t>Math Methods: Ch. 8 (Vector Calculus)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1633,18 +1629,22 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Centrifugal force; Coriolis force</t>
+          <t>Angular velocity; rotating frames</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>9.6-9.8</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr"/>
+          <t>9.3-9.5</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Math Methods: Ch. 8 (Vectors in Curvilinear Coordinates)</t>
+        </is>
+      </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>9.12</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr"/>
@@ -1664,63 +1664,59 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
+          <t>Centrifugal force; Coriolis force</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>9.6-9.8</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>9.12</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>HW10 (Ch 8)</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Mon Nov 23</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
           <t>Coupled oscillators; two masses and three springs</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>11.1-11.2</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>Knight: Ch. 15 (Oscillations)
 Math Methods: Ch. 6 (Eigenvectors/Eigenvalues)
 Review the ideas behind basis vectors</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>11.1</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>HW10 (Ch 8)</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B35" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Mon Nov 23</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>Normal coordinates; weakly coupled oscillators; start the double pendulum</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>11.2-11.4</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>Math Methods: Ch. 6 (Eigenvectors/Eigenvalues)</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>Read 11.3: in a sentence or two, what happens to the energy of two weakly coupled pendulums over time?</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr"/>
@@ -1778,18 +1774,22 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Double pendulum</t>
+          <t>Normal coordinates; weakly coupled oscillators; start the double pendulum</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>11.4</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr"/>
+          <t>11.2-11.4</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Math Methods: Ch. 6 (Eigenvectors/Eigenvalues)</t>
+        </is>
+      </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Write down the Lagrangian of a simple pendulum (length L, angle phi); no need to solve it</t>
+          <t>Read 11.3: in a sentence or two, what happens to the energy of two weakly coupled pendulums over time?</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -1813,18 +1813,18 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Chaos: the driven damped pendulum; period doubling</t>
+          <t>Double pendulum</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>12.1-12.4</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr"/>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Read 12.1-12.2: in a sentence, what does it mean for an equation of motion to be linear, and what do we lose when it isn't?</t>
+          <t>Write down the Lagrangian of a simple pendulum (length L, angle phi); no need to solve it</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -1844,18 +1844,18 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Chaos: sensitivity to initial conditions; Liouville aside [BRING LAPTOP]</t>
+          <t>Chaos: the driven damped pendulum; period doubling [BRING LAPTOP]</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>12.4-12.5</t>
+          <t>12.1-12.4</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Log into jupyterhub.smith.edu and open the driven-pendulum notebook on Moodle; bring your laptop</t>
+          <t>Read 12.1-12.2: in a sentence, what does it mean for an equation of motion to be linear, and what do we lose when it isn't?</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -1906,12 +1906,20 @@
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Flex day: Noether's theorem (Taylor 7.8) OR Jarzynski OR catch-up</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr"/>
+          <t>Chaos: sensitivity to initial conditions; Liouville aside</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>12.4-12.5</t>
+        </is>
+      </c>
       <c r="F42" s="5" t="inlineStr"/>
-      <c r="G42" s="5" t="inlineStr"/>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>Log into jupyterhub.smith.edu and open the driven-pendulum notebook on Moodle; bring your laptop</t>
+        </is>
+      </c>
       <c r="H42" s="5" t="inlineStr"/>
       <c r="I42" s="5" t="inlineStr"/>
     </row>

</xml_diff>